<commit_message>
Backend endpoints for country-scenario management
Implemented POST and DELETE endpoints with updated logic to modify the COUNTRIES list in config.py

TODO: Implement logic to duplicate the templates folder when a country is added
</commit_message>
<xml_diff>
--- a/backend/{templates}/capex-fuels-{model}.xlsx
+++ b/backend/{templates}/capex-fuels-{model}.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{76E76D21-28F7-4F66-BCD5-940D1BD49D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB556B36-7A8C-413D-A39D-8998723FD2C8}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{76E76D21-28F7-4F66-BCD5-940D1BD49D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CC36D45-65FC-45BD-829C-9AA1F11771B9}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="6" r:id="rId1"/>
@@ -264,6 +264,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Manage fuels and models per country-scenario in redesigned sidebar
Enabled add/remove functionality for fuels in the Financial Inputs section

Adopted same pattern as country scenarios: new entry in config.py

Created per-country dictionary storing fuel lists by section (e.g., Financial Inputs, Financial Statements)

Distinction made between fuel types per section (e.g., ecooking, just access, electricity)

Started handling techno-economic scenario management

Created per-country dictionary storing techno-economic models

Added dictionary to store year range for each scenario, defined when BAU model is created

Year range must remain consistent throughout the scenario
</commit_message>
<xml_diff>
--- a/backend/{templates}/capex-fuels-{model}.xlsx
+++ b/backend/{templates}/capex-fuels-{model}.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{76E76D21-28F7-4F66-BCD5-940D1BD49D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CC36D45-65FC-45BD-829C-9AA1F11771B9}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{76E76D21-28F7-4F66-BCD5-940D1BD49D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E1BEAE6-E1D9-445A-94A6-510FE10800A8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="24">
   <si>
     <t>Units</t>
   </si>
@@ -533,13 +533,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF4224F1-5D48-4FE4-980F-718DB45087F0}">
-  <dimension ref="A1:AS18"/>
+  <dimension ref="A1:AR18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="33.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -553,130 +553,127 @@
         <v>1</v>
       </c>
       <c r="E1" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F1" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G1" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H1" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I1" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="J1" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K1" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="L1" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="M1" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="N1" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="O1" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="P1" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="Q1" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="R1" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="S1" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="T1" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="U1" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="V1" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="W1" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="X1" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="Y1" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Z1" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="AA1" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AB1" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AC1" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AD1" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AE1" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AF1" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AG1" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AH1" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AI1" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AJ1" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AK1" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AL1" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AM1" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AN1" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AO1" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AP1" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AQ1" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AR1" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AS1" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>16</v>
       </c>
@@ -809,11 +806,8 @@
       <c r="AR2" s="7">
         <v>0</v>
       </c>
-      <c r="AS2" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="3" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>16</v>
       </c>
@@ -946,11 +940,8 @@
       <c r="AR3" s="7">
         <v>0</v>
       </c>
-      <c r="AS3" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="4" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
@@ -1083,11 +1074,8 @@
       <c r="AR4" s="7">
         <v>0</v>
       </c>
-      <c r="AS4" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>16</v>
       </c>
@@ -1220,11 +1208,8 @@
       <c r="AR5" s="7">
         <v>0</v>
       </c>
-      <c r="AS5" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="6" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
@@ -1357,11 +1342,8 @@
       <c r="AR6" s="7">
         <v>0</v>
       </c>
-      <c r="AS6" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="7" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>16</v>
       </c>
@@ -1494,11 +1476,8 @@
       <c r="AR7" s="7">
         <v>0</v>
       </c>
-      <c r="AS7" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="8" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>16</v>
       </c>
@@ -1631,11 +1610,8 @@
       <c r="AR8" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AS8" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="9" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
@@ -1768,11 +1744,8 @@
       <c r="AR9" s="7">
         <v>0</v>
       </c>
-      <c r="AS9" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -1786,130 +1759,127 @@
         <v>1</v>
       </c>
       <c r="E10" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F10" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G10" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H10" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I10" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="J10" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K10" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="L10" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="M10" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="N10" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="O10" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="P10" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="Q10" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="R10" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="S10" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="T10" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="U10" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="V10" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="W10" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="X10" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="Y10" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Z10" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="AA10" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AB10" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AC10" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AD10" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AE10" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AF10" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AG10" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AH10" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AI10" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AJ10" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AK10" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AL10" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AM10" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AN10" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AO10" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AP10" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AQ10" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AR10" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AS10" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="11" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -2042,11 +2012,8 @@
       <c r="AR11" s="7">
         <v>0</v>
       </c>
-      <c r="AS11" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="12" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -2179,11 +2146,8 @@
       <c r="AR12" s="7">
         <v>0</v>
       </c>
-      <c r="AS12" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="13" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -2316,11 +2280,8 @@
       <c r="AR13" s="7">
         <v>0</v>
       </c>
-      <c r="AS13" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="14" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
@@ -2453,11 +2414,8 @@
       <c r="AR14" s="7">
         <v>0</v>
       </c>
-      <c r="AS14" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="15" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>17</v>
       </c>
@@ -2590,11 +2548,8 @@
       <c r="AR15" s="7">
         <v>0</v>
       </c>
-      <c r="AS15" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="16" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -2727,11 +2682,8 @@
       <c r="AR16" s="7">
         <v>0</v>
       </c>
-      <c r="AS16" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="17" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
@@ -2864,11 +2816,8 @@
       <c r="AR17" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AS17" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="18" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
@@ -2999,9 +2948,6 @@
         <v>0</v>
       </c>
       <c r="AR18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AS18" s="7">
         <v>0</v>
       </c>
     </row>
@@ -3013,14 +2959,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:AS27"/>
+  <dimension ref="A1:AR27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -3034,130 +2980,127 @@
         <v>1</v>
       </c>
       <c r="E1" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F1" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G1" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H1" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I1" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="J1" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K1" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="L1" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="M1" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="N1" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="O1" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="P1" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="Q1" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="R1" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="S1" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="T1" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="U1" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="V1" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="W1" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="X1" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="Y1" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Z1" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="AA1" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AB1" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AC1" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AD1" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AE1" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AF1" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AG1" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AH1" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AI1" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AJ1" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AK1" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AL1" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AM1" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AN1" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AO1" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AP1" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AQ1" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AR1" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AS1" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
@@ -3290,11 +3233,8 @@
       <c r="AR2" s="7">
         <v>0</v>
       </c>
-      <c r="AS2" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="3" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>18</v>
       </c>
@@ -3427,11 +3367,8 @@
       <c r="AR3" s="7">
         <v>0</v>
       </c>
-      <c r="AS3" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="4" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>18</v>
       </c>
@@ -3564,11 +3501,8 @@
       <c r="AR4" s="7">
         <v>0</v>
       </c>
-      <c r="AS4" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
@@ -3701,11 +3635,8 @@
       <c r="AR5" s="7">
         <v>0</v>
       </c>
-      <c r="AS5" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="6" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>18</v>
       </c>
@@ -3838,11 +3769,8 @@
       <c r="AR6" s="7">
         <v>0</v>
       </c>
-      <c r="AS6" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="7" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
@@ -3975,11 +3903,8 @@
       <c r="AR7" s="7">
         <v>0</v>
       </c>
-      <c r="AS7" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="8" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
@@ -4112,11 +4037,8 @@
       <c r="AR8" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AS8" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="9" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>18</v>
       </c>
@@ -4249,11 +4171,8 @@
       <c r="AR9" s="7">
         <v>0</v>
       </c>
-      <c r="AS9" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -4267,130 +4186,127 @@
         <v>1</v>
       </c>
       <c r="E10" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F10" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G10" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H10" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I10" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="J10" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K10" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="L10" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="M10" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="N10" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="O10" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="P10" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="Q10" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="R10" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="S10" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="T10" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="U10" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="V10" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="W10" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="X10" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="Y10" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Z10" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="AA10" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AB10" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AC10" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AD10" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AE10" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AF10" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AG10" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AH10" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AI10" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AJ10" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AK10" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AL10" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AM10" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AN10" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AO10" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AP10" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AQ10" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AR10" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AS10" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="11" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>19</v>
       </c>
@@ -4523,11 +4439,8 @@
       <c r="AR11" s="7">
         <v>0</v>
       </c>
-      <c r="AS11" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="12" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>19</v>
       </c>
@@ -4660,11 +4573,8 @@
       <c r="AR12" s="7">
         <v>0</v>
       </c>
-      <c r="AS12" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="13" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>19</v>
       </c>
@@ -4797,11 +4707,8 @@
       <c r="AR13" s="7">
         <v>0</v>
       </c>
-      <c r="AS13" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="14" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>19</v>
       </c>
@@ -4934,11 +4841,8 @@
       <c r="AR14" s="7">
         <v>0</v>
       </c>
-      <c r="AS14" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="15" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>19</v>
       </c>
@@ -5071,11 +4975,8 @@
       <c r="AR15" s="7">
         <v>0</v>
       </c>
-      <c r="AS15" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="16" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>19</v>
       </c>
@@ -5208,11 +5109,8 @@
       <c r="AR16" s="7">
         <v>0</v>
       </c>
-      <c r="AS16" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="17" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>19</v>
       </c>
@@ -5345,11 +5243,8 @@
       <c r="AR17" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AS17" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="18" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
@@ -5482,11 +5377,8 @@
       <c r="AR18" s="7">
         <v>0</v>
       </c>
-      <c r="AS18" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="19" spans="1:45" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>23</v>
       </c>
@@ -5500,130 +5392,127 @@
         <v>1</v>
       </c>
       <c r="E19" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F19" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G19" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H19" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I19" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="J19" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="K19" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="L19" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="M19" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="N19" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="O19" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="P19" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="Q19" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="R19" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="S19" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="T19" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="U19" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="V19" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="W19" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="X19" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="Y19" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Z19" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="AA19" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AB19" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AC19" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AD19" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AE19" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AF19" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AG19" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AH19" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AI19" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AJ19" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AK19" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AL19" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AM19" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AN19" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AO19" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AP19" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AQ19" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AR19" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AS19" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="20" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>20</v>
       </c>
@@ -5756,11 +5645,8 @@
       <c r="AR20" s="7">
         <v>0</v>
       </c>
-      <c r="AS20" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="21" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>20</v>
       </c>
@@ -5893,11 +5779,8 @@
       <c r="AR21" s="7">
         <v>0</v>
       </c>
-      <c r="AS21" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="22" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>20</v>
       </c>
@@ -6030,11 +5913,8 @@
       <c r="AR22" s="7">
         <v>0</v>
       </c>
-      <c r="AS22" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="23" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>20</v>
       </c>
@@ -6167,11 +6047,8 @@
       <c r="AR23" s="7">
         <v>0</v>
       </c>
-      <c r="AS23" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="24" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>20</v>
       </c>
@@ -6304,11 +6181,8 @@
       <c r="AR24" s="7">
         <v>0</v>
       </c>
-      <c r="AS24" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="25" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
         <v>20</v>
       </c>
@@ -6441,11 +6315,8 @@
       <c r="AR25" s="7">
         <v>0</v>
       </c>
-      <c r="AS25" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="26" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
         <v>20</v>
       </c>
@@ -6578,11 +6449,8 @@
       <c r="AR26" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AS26" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="27" spans="1:45" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
         <v>20</v>
       </c>
@@ -6713,9 +6581,6 @@
         <v>0</v>
       </c>
       <c r="AR27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AS27" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor and feature expansion
- Restructured the user input template for uploading data: removed separation between local and upstream for fuels (e.g. LPG) and simplified the electricity inputs by getting rid of e-heating while keeping grid/off-grid distinction.

- Updated LPG as the default example fuel template with unified CAPEX/OPEX.

- Added new input fields: demand, tariff, and upstream cost for each fuel type (electricity grid and off-grid), reflected in both backend templates and UI.

- Added backend and UI logic to define consumer types per model in the model management tab (currently hidden for future extensions).

- Extended BAU model inputs to include demand, tariff, upstream, CAPEX, and OPEX, enabling proper comparisons with other models. Added a new "Technoeconomic Inputs" tab in the sidebar.

- Updated scenario creation to request tax rate and inflation, stored in backend `config.json` per country/model/fuel.
</commit_message>
<xml_diff>
--- a/backend/{templates}/capex-fuels-{model}.xlsx
+++ b/backend/{templates}/capex-fuels-{model}.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarr\OneDrive\Escritorio\IIT\CC-WBT\backend\{templates}\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{76E76D21-28F7-4F66-BCD5-940D1BD49D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E1BEAE6-E1D9-445A-94A6-510FE10800A8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E2BDE7-11A9-429F-9E0E-82D55F13BE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="18">
   <si>
     <t>Units</t>
   </si>
@@ -72,34 +72,10 @@
     <t>Acc. Total CAPEX</t>
   </si>
   <si>
-    <t>Local Processing</t>
-  </si>
-  <si>
-    <t>Local Transport</t>
-  </si>
-  <si>
-    <t>Upstream</t>
-  </si>
-  <si>
     <t>Grid</t>
   </si>
   <si>
     <t>Off-Grid</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>O-G</t>
-  </si>
-  <si>
-    <t>LP</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>U</t>
   </si>
   <si>
     <t>Maintenance CAPEX</t>
@@ -109,6 +85,12 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>GRID</t>
+  </si>
+  <si>
+    <t>OFF-GRID</t>
   </si>
 </sst>
 </file>
@@ -264,10 +246,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -541,10 +519,10 @@
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -946,7 +924,7 @@
         <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>2</v>
@@ -1080,7 +1058,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>2</v>
@@ -1747,10 +1725,10 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>0</v>
@@ -2152,7 +2130,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>2</v>
@@ -2286,7 +2264,7 @@
         <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>2</v>
@@ -2959,157 +2937,154 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:AR27"/>
+  <dimension ref="A1:AQ9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
+      <c r="D1" s="5">
+        <v>2021</v>
+      </c>
       <c r="E1" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F1" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="G1" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="H1" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="I1" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="J1" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="K1" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="L1" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="M1" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="N1" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="O1" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="P1" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="Q1" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="R1" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="S1" s="5">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="T1" s="5">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="U1" s="5">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="V1" s="5">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="W1" s="5">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="X1" s="5">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="Y1" s="5">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="Z1" s="5">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="AA1" s="5">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="AB1" s="5">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AC1" s="5">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AD1" s="5">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AE1" s="5">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AF1" s="5">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AG1" s="5">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="AH1" s="5">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="AI1" s="5">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="AJ1" s="5">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="AK1" s="5">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="AL1" s="5">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="AM1" s="5">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="AN1" s="5">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="AO1" s="5">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="AP1" s="5">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="AQ1" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AR1" s="5">
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C2" s="7">
+        <v>0</v>
+      </c>
       <c r="D2" s="7">
         <v>0</v>
       </c>
@@ -3230,20 +3205,17 @@
       <c r="AQ2" s="7">
         <v>0</v>
       </c>
-      <c r="AR2" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="3" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C3" s="7">
+        <v>0</v>
+      </c>
       <c r="D3" s="7">
         <v>0</v>
       </c>
@@ -3364,20 +3336,17 @@
       <c r="AQ3" s="7">
         <v>0</v>
       </c>
-      <c r="AR3" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="4" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="6" t="s">
+    <row r="4" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C4" s="7">
+        <v>0</v>
+      </c>
       <c r="D4" s="7">
         <v>0</v>
       </c>
@@ -3498,20 +3467,17 @@
       <c r="AQ4" s="7">
         <v>0</v>
       </c>
-      <c r="AR4" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="6" t="s">
+    <row r="5" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C5" s="7">
+        <v>0</v>
+      </c>
       <c r="D5" s="7">
         <v>0</v>
       </c>
@@ -3632,20 +3598,17 @@
       <c r="AQ5" s="7">
         <v>0</v>
       </c>
-      <c r="AR5" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="6" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    <row r="6" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="B6" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
       <c r="D6" s="7">
         <v>0</v>
       </c>
@@ -3766,20 +3729,17 @@
       <c r="AQ6" s="7">
         <v>0</v>
       </c>
-      <c r="AR6" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="7" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="7" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C7" s="7">
+        <v>0</v>
+      </c>
       <c r="D7" s="7">
         <v>0</v>
       </c>
@@ -3900,22 +3860,19 @@
       <c r="AQ7" s="7">
         <v>0</v>
       </c>
-      <c r="AR7" s="7">
-        <v>0</v>
-      </c>
     </row>
-    <row r="8" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="7">
-        <v>0</v>
+      <c r="C8" s="7">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>3</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>3</v>
@@ -4034,20 +3991,17 @@
       <c r="AQ8" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="AR8" s="8" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="9" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="9" spans="1:43" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="C9" s="7">
+        <v>0</v>
+      </c>
       <c r="D9" s="7">
         <v>0</v>
       </c>
@@ -4166,2421 +4120,6 @@
         <v>0</v>
       </c>
       <c r="AQ9" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR9" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5">
-        <v>2021</v>
-      </c>
-      <c r="F10" s="5">
-        <v>2022</v>
-      </c>
-      <c r="G10" s="5">
-        <v>2023</v>
-      </c>
-      <c r="H10" s="5">
-        <v>2024</v>
-      </c>
-      <c r="I10" s="5">
-        <v>2025</v>
-      </c>
-      <c r="J10" s="5">
-        <v>2026</v>
-      </c>
-      <c r="K10" s="5">
-        <v>2027</v>
-      </c>
-      <c r="L10" s="5">
-        <v>2028</v>
-      </c>
-      <c r="M10" s="5">
-        <v>2029</v>
-      </c>
-      <c r="N10" s="5">
-        <v>2030</v>
-      </c>
-      <c r="O10" s="5">
-        <v>2031</v>
-      </c>
-      <c r="P10" s="5">
-        <v>2032</v>
-      </c>
-      <c r="Q10" s="5">
-        <v>2033</v>
-      </c>
-      <c r="R10" s="5">
-        <v>2034</v>
-      </c>
-      <c r="S10" s="5">
-        <v>2035</v>
-      </c>
-      <c r="T10" s="5">
-        <v>2036</v>
-      </c>
-      <c r="U10" s="5">
-        <v>2037</v>
-      </c>
-      <c r="V10" s="5">
-        <v>2038</v>
-      </c>
-      <c r="W10" s="5">
-        <v>2039</v>
-      </c>
-      <c r="X10" s="5">
-        <v>2040</v>
-      </c>
-      <c r="Y10" s="5">
-        <v>2041</v>
-      </c>
-      <c r="Z10" s="5">
-        <v>2042</v>
-      </c>
-      <c r="AA10" s="5">
-        <v>2043</v>
-      </c>
-      <c r="AB10" s="5">
-        <v>2044</v>
-      </c>
-      <c r="AC10" s="5">
-        <v>2045</v>
-      </c>
-      <c r="AD10" s="5">
-        <v>2046</v>
-      </c>
-      <c r="AE10" s="5">
-        <v>2047</v>
-      </c>
-      <c r="AF10" s="5">
-        <v>2048</v>
-      </c>
-      <c r="AG10" s="5">
-        <v>2049</v>
-      </c>
-      <c r="AH10" s="5">
-        <v>2050</v>
-      </c>
-      <c r="AI10" s="5">
-        <v>2051</v>
-      </c>
-      <c r="AJ10" s="5">
-        <v>2052</v>
-      </c>
-      <c r="AK10" s="5">
-        <v>2053</v>
-      </c>
-      <c r="AL10" s="5">
-        <v>2054</v>
-      </c>
-      <c r="AM10" s="5">
-        <v>2055</v>
-      </c>
-      <c r="AN10" s="5">
-        <v>2056</v>
-      </c>
-      <c r="AO10" s="5">
-        <v>2057</v>
-      </c>
-      <c r="AP10" s="5">
-        <v>2058</v>
-      </c>
-      <c r="AQ10" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AR10" s="5">
-        <v>2060</v>
-      </c>
-    </row>
-    <row r="11" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7">
-        <v>0</v>
-      </c>
-      <c r="F11" s="7">
-        <v>0</v>
-      </c>
-      <c r="G11" s="7">
-        <v>0</v>
-      </c>
-      <c r="H11" s="7">
-        <v>0</v>
-      </c>
-      <c r="I11" s="7">
-        <v>0</v>
-      </c>
-      <c r="J11" s="7">
-        <v>0</v>
-      </c>
-      <c r="K11" s="7">
-        <v>0</v>
-      </c>
-      <c r="L11" s="7">
-        <v>0</v>
-      </c>
-      <c r="M11" s="7">
-        <v>0</v>
-      </c>
-      <c r="N11" s="7">
-        <v>0</v>
-      </c>
-      <c r="O11" s="7">
-        <v>0</v>
-      </c>
-      <c r="P11" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="7">
-        <v>0</v>
-      </c>
-      <c r="R11" s="7">
-        <v>0</v>
-      </c>
-      <c r="S11" s="7">
-        <v>0</v>
-      </c>
-      <c r="T11" s="7">
-        <v>0</v>
-      </c>
-      <c r="U11" s="7">
-        <v>0</v>
-      </c>
-      <c r="V11" s="7">
-        <v>0</v>
-      </c>
-      <c r="W11" s="7">
-        <v>0</v>
-      </c>
-      <c r="X11" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ11" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR11" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="7">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7">
-        <v>0</v>
-      </c>
-      <c r="H12" s="7">
-        <v>0</v>
-      </c>
-      <c r="I12" s="7">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7">
-        <v>0</v>
-      </c>
-      <c r="K12" s="7">
-        <v>0</v>
-      </c>
-      <c r="L12" s="7">
-        <v>0</v>
-      </c>
-      <c r="M12" s="7">
-        <v>0</v>
-      </c>
-      <c r="N12" s="7">
-        <v>0</v>
-      </c>
-      <c r="O12" s="7">
-        <v>0</v>
-      </c>
-      <c r="P12" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="7">
-        <v>0</v>
-      </c>
-      <c r="R12" s="7">
-        <v>0</v>
-      </c>
-      <c r="S12" s="7">
-        <v>0</v>
-      </c>
-      <c r="T12" s="7">
-        <v>0</v>
-      </c>
-      <c r="U12" s="7">
-        <v>0</v>
-      </c>
-      <c r="V12" s="7">
-        <v>0</v>
-      </c>
-      <c r="W12" s="7">
-        <v>0</v>
-      </c>
-      <c r="X12" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR12" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D13" s="7">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7">
-        <v>0</v>
-      </c>
-      <c r="H13" s="7">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7">
-        <v>0</v>
-      </c>
-      <c r="K13" s="7">
-        <v>0</v>
-      </c>
-      <c r="L13" s="7">
-        <v>0</v>
-      </c>
-      <c r="M13" s="7">
-        <v>0</v>
-      </c>
-      <c r="N13" s="7">
-        <v>0</v>
-      </c>
-      <c r="O13" s="7">
-        <v>0</v>
-      </c>
-      <c r="P13" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="7">
-        <v>0</v>
-      </c>
-      <c r="R13" s="7">
-        <v>0</v>
-      </c>
-      <c r="S13" s="7">
-        <v>0</v>
-      </c>
-      <c r="T13" s="7">
-        <v>0</v>
-      </c>
-      <c r="U13" s="7">
-        <v>0</v>
-      </c>
-      <c r="V13" s="7">
-        <v>0</v>
-      </c>
-      <c r="W13" s="7">
-        <v>0</v>
-      </c>
-      <c r="X13" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ13" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR13" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="7">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7">
-        <v>0</v>
-      </c>
-      <c r="K14" s="7">
-        <v>0</v>
-      </c>
-      <c r="L14" s="7">
-        <v>0</v>
-      </c>
-      <c r="M14" s="7">
-        <v>0</v>
-      </c>
-      <c r="N14" s="7">
-        <v>0</v>
-      </c>
-      <c r="O14" s="7">
-        <v>0</v>
-      </c>
-      <c r="P14" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="7">
-        <v>0</v>
-      </c>
-      <c r="R14" s="7">
-        <v>0</v>
-      </c>
-      <c r="S14" s="7">
-        <v>0</v>
-      </c>
-      <c r="T14" s="7">
-        <v>0</v>
-      </c>
-      <c r="U14" s="7">
-        <v>0</v>
-      </c>
-      <c r="V14" s="7">
-        <v>0</v>
-      </c>
-      <c r="W14" s="7">
-        <v>0</v>
-      </c>
-      <c r="X14" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ14" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR14" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
-        <v>0</v>
-      </c>
-      <c r="G15" s="7">
-        <v>0</v>
-      </c>
-      <c r="H15" s="7">
-        <v>0</v>
-      </c>
-      <c r="I15" s="7">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7">
-        <v>0</v>
-      </c>
-      <c r="K15" s="7">
-        <v>0</v>
-      </c>
-      <c r="L15" s="7">
-        <v>0</v>
-      </c>
-      <c r="M15" s="7">
-        <v>0</v>
-      </c>
-      <c r="N15" s="7">
-        <v>0</v>
-      </c>
-      <c r="O15" s="7">
-        <v>0</v>
-      </c>
-      <c r="P15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="7">
-        <v>0</v>
-      </c>
-      <c r="R15" s="7">
-        <v>0</v>
-      </c>
-      <c r="S15" s="7">
-        <v>0</v>
-      </c>
-      <c r="T15" s="7">
-        <v>0</v>
-      </c>
-      <c r="U15" s="7">
-        <v>0</v>
-      </c>
-      <c r="V15" s="7">
-        <v>0</v>
-      </c>
-      <c r="W15" s="7">
-        <v>0</v>
-      </c>
-      <c r="X15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ15" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR15" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D16" s="7">
-        <v>0</v>
-      </c>
-      <c r="E16" s="7">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7">
-        <v>0</v>
-      </c>
-      <c r="G16" s="7">
-        <v>0</v>
-      </c>
-      <c r="H16" s="7">
-        <v>0</v>
-      </c>
-      <c r="I16" s="7">
-        <v>0</v>
-      </c>
-      <c r="J16" s="7">
-        <v>0</v>
-      </c>
-      <c r="K16" s="7">
-        <v>0</v>
-      </c>
-      <c r="L16" s="7">
-        <v>0</v>
-      </c>
-      <c r="M16" s="7">
-        <v>0</v>
-      </c>
-      <c r="N16" s="7">
-        <v>0</v>
-      </c>
-      <c r="O16" s="7">
-        <v>0</v>
-      </c>
-      <c r="P16" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="7">
-        <v>0</v>
-      </c>
-      <c r="R16" s="7">
-        <v>0</v>
-      </c>
-      <c r="S16" s="7">
-        <v>0</v>
-      </c>
-      <c r="T16" s="7">
-        <v>0</v>
-      </c>
-      <c r="U16" s="7">
-        <v>0</v>
-      </c>
-      <c r="V16" s="7">
-        <v>0</v>
-      </c>
-      <c r="W16" s="7">
-        <v>0</v>
-      </c>
-      <c r="X16" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ16" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR16" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="7">
-        <v>0</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="N17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="O17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="P17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="R17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="S17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="T17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="U17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="V17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="W17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="X17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AQ17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR17" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="7">
-        <v>0</v>
-      </c>
-      <c r="E18" s="7">
-        <v>0</v>
-      </c>
-      <c r="F18" s="7">
-        <v>0</v>
-      </c>
-      <c r="G18" s="7">
-        <v>0</v>
-      </c>
-      <c r="H18" s="7">
-        <v>0</v>
-      </c>
-      <c r="I18" s="7">
-        <v>0</v>
-      </c>
-      <c r="J18" s="7">
-        <v>0</v>
-      </c>
-      <c r="K18" s="7">
-        <v>0</v>
-      </c>
-      <c r="L18" s="7">
-        <v>0</v>
-      </c>
-      <c r="M18" s="7">
-        <v>0</v>
-      </c>
-      <c r="N18" s="7">
-        <v>0</v>
-      </c>
-      <c r="O18" s="7">
-        <v>0</v>
-      </c>
-      <c r="P18" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="7">
-        <v>0</v>
-      </c>
-      <c r="R18" s="7">
-        <v>0</v>
-      </c>
-      <c r="S18" s="7">
-        <v>0</v>
-      </c>
-      <c r="T18" s="7">
-        <v>0</v>
-      </c>
-      <c r="U18" s="7">
-        <v>0</v>
-      </c>
-      <c r="V18" s="7">
-        <v>0</v>
-      </c>
-      <c r="W18" s="7">
-        <v>0</v>
-      </c>
-      <c r="X18" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ18" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR18" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E19" s="5">
-        <v>2021</v>
-      </c>
-      <c r="F19" s="5">
-        <v>2022</v>
-      </c>
-      <c r="G19" s="5">
-        <v>2023</v>
-      </c>
-      <c r="H19" s="5">
-        <v>2024</v>
-      </c>
-      <c r="I19" s="5">
-        <v>2025</v>
-      </c>
-      <c r="J19" s="5">
-        <v>2026</v>
-      </c>
-      <c r="K19" s="5">
-        <v>2027</v>
-      </c>
-      <c r="L19" s="5">
-        <v>2028</v>
-      </c>
-      <c r="M19" s="5">
-        <v>2029</v>
-      </c>
-      <c r="N19" s="5">
-        <v>2030</v>
-      </c>
-      <c r="O19" s="5">
-        <v>2031</v>
-      </c>
-      <c r="P19" s="5">
-        <v>2032</v>
-      </c>
-      <c r="Q19" s="5">
-        <v>2033</v>
-      </c>
-      <c r="R19" s="5">
-        <v>2034</v>
-      </c>
-      <c r="S19" s="5">
-        <v>2035</v>
-      </c>
-      <c r="T19" s="5">
-        <v>2036</v>
-      </c>
-      <c r="U19" s="5">
-        <v>2037</v>
-      </c>
-      <c r="V19" s="5">
-        <v>2038</v>
-      </c>
-      <c r="W19" s="5">
-        <v>2039</v>
-      </c>
-      <c r="X19" s="5">
-        <v>2040</v>
-      </c>
-      <c r="Y19" s="5">
-        <v>2041</v>
-      </c>
-      <c r="Z19" s="5">
-        <v>2042</v>
-      </c>
-      <c r="AA19" s="5">
-        <v>2043</v>
-      </c>
-      <c r="AB19" s="5">
-        <v>2044</v>
-      </c>
-      <c r="AC19" s="5">
-        <v>2045</v>
-      </c>
-      <c r="AD19" s="5">
-        <v>2046</v>
-      </c>
-      <c r="AE19" s="5">
-        <v>2047</v>
-      </c>
-      <c r="AF19" s="5">
-        <v>2048</v>
-      </c>
-      <c r="AG19" s="5">
-        <v>2049</v>
-      </c>
-      <c r="AH19" s="5">
-        <v>2050</v>
-      </c>
-      <c r="AI19" s="5">
-        <v>2051</v>
-      </c>
-      <c r="AJ19" s="5">
-        <v>2052</v>
-      </c>
-      <c r="AK19" s="5">
-        <v>2053</v>
-      </c>
-      <c r="AL19" s="5">
-        <v>2054</v>
-      </c>
-      <c r="AM19" s="5">
-        <v>2055</v>
-      </c>
-      <c r="AN19" s="5">
-        <v>2056</v>
-      </c>
-      <c r="AO19" s="5">
-        <v>2057</v>
-      </c>
-      <c r="AP19" s="5">
-        <v>2058</v>
-      </c>
-      <c r="AQ19" s="5">
-        <v>2059</v>
-      </c>
-      <c r="AR19" s="5">
-        <v>2060</v>
-      </c>
-    </row>
-    <row r="20" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="7">
-        <v>0</v>
-      </c>
-      <c r="E20" s="7">
-        <v>0</v>
-      </c>
-      <c r="F20" s="7">
-        <v>0</v>
-      </c>
-      <c r="G20" s="7">
-        <v>0</v>
-      </c>
-      <c r="H20" s="7">
-        <v>0</v>
-      </c>
-      <c r="I20" s="7">
-        <v>0</v>
-      </c>
-      <c r="J20" s="7">
-        <v>0</v>
-      </c>
-      <c r="K20" s="7">
-        <v>0</v>
-      </c>
-      <c r="L20" s="7">
-        <v>0</v>
-      </c>
-      <c r="M20" s="7">
-        <v>0</v>
-      </c>
-      <c r="N20" s="7">
-        <v>0</v>
-      </c>
-      <c r="O20" s="7">
-        <v>0</v>
-      </c>
-      <c r="P20" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="7">
-        <v>0</v>
-      </c>
-      <c r="R20" s="7">
-        <v>0</v>
-      </c>
-      <c r="S20" s="7">
-        <v>0</v>
-      </c>
-      <c r="T20" s="7">
-        <v>0</v>
-      </c>
-      <c r="U20" s="7">
-        <v>0</v>
-      </c>
-      <c r="V20" s="7">
-        <v>0</v>
-      </c>
-      <c r="W20" s="7">
-        <v>0</v>
-      </c>
-      <c r="X20" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ20" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR20" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="7">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7">
-        <v>0</v>
-      </c>
-      <c r="F21" s="7">
-        <v>0</v>
-      </c>
-      <c r="G21" s="7">
-        <v>0</v>
-      </c>
-      <c r="H21" s="7">
-        <v>0</v>
-      </c>
-      <c r="I21" s="7">
-        <v>0</v>
-      </c>
-      <c r="J21" s="7">
-        <v>0</v>
-      </c>
-      <c r="K21" s="7">
-        <v>0</v>
-      </c>
-      <c r="L21" s="7">
-        <v>0</v>
-      </c>
-      <c r="M21" s="7">
-        <v>0</v>
-      </c>
-      <c r="N21" s="7">
-        <v>0</v>
-      </c>
-      <c r="O21" s="7">
-        <v>0</v>
-      </c>
-      <c r="P21" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="7">
-        <v>0</v>
-      </c>
-      <c r="R21" s="7">
-        <v>0</v>
-      </c>
-      <c r="S21" s="7">
-        <v>0</v>
-      </c>
-      <c r="T21" s="7">
-        <v>0</v>
-      </c>
-      <c r="U21" s="7">
-        <v>0</v>
-      </c>
-      <c r="V21" s="7">
-        <v>0</v>
-      </c>
-      <c r="W21" s="7">
-        <v>0</v>
-      </c>
-      <c r="X21" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ21" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR21" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="7">
-        <v>0</v>
-      </c>
-      <c r="E22" s="7">
-        <v>0</v>
-      </c>
-      <c r="F22" s="7">
-        <v>0</v>
-      </c>
-      <c r="G22" s="7">
-        <v>0</v>
-      </c>
-      <c r="H22" s="7">
-        <v>0</v>
-      </c>
-      <c r="I22" s="7">
-        <v>0</v>
-      </c>
-      <c r="J22" s="7">
-        <v>0</v>
-      </c>
-      <c r="K22" s="7">
-        <v>0</v>
-      </c>
-      <c r="L22" s="7">
-        <v>0</v>
-      </c>
-      <c r="M22" s="7">
-        <v>0</v>
-      </c>
-      <c r="N22" s="7">
-        <v>0</v>
-      </c>
-      <c r="O22" s="7">
-        <v>0</v>
-      </c>
-      <c r="P22" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="7">
-        <v>0</v>
-      </c>
-      <c r="R22" s="7">
-        <v>0</v>
-      </c>
-      <c r="S22" s="7">
-        <v>0</v>
-      </c>
-      <c r="T22" s="7">
-        <v>0</v>
-      </c>
-      <c r="U22" s="7">
-        <v>0</v>
-      </c>
-      <c r="V22" s="7">
-        <v>0</v>
-      </c>
-      <c r="W22" s="7">
-        <v>0</v>
-      </c>
-      <c r="X22" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ22" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR22" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D23" s="7">
-        <v>0</v>
-      </c>
-      <c r="E23" s="7">
-        <v>0</v>
-      </c>
-      <c r="F23" s="7">
-        <v>0</v>
-      </c>
-      <c r="G23" s="7">
-        <v>0</v>
-      </c>
-      <c r="H23" s="7">
-        <v>0</v>
-      </c>
-      <c r="I23" s="7">
-        <v>0</v>
-      </c>
-      <c r="J23" s="7">
-        <v>0</v>
-      </c>
-      <c r="K23" s="7">
-        <v>0</v>
-      </c>
-      <c r="L23" s="7">
-        <v>0</v>
-      </c>
-      <c r="M23" s="7">
-        <v>0</v>
-      </c>
-      <c r="N23" s="7">
-        <v>0</v>
-      </c>
-      <c r="O23" s="7">
-        <v>0</v>
-      </c>
-      <c r="P23" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="7">
-        <v>0</v>
-      </c>
-      <c r="R23" s="7">
-        <v>0</v>
-      </c>
-      <c r="S23" s="7">
-        <v>0</v>
-      </c>
-      <c r="T23" s="7">
-        <v>0</v>
-      </c>
-      <c r="U23" s="7">
-        <v>0</v>
-      </c>
-      <c r="V23" s="7">
-        <v>0</v>
-      </c>
-      <c r="W23" s="7">
-        <v>0</v>
-      </c>
-      <c r="X23" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ23" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR23" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="7">
-        <v>0</v>
-      </c>
-      <c r="E24" s="7">
-        <v>0</v>
-      </c>
-      <c r="F24" s="7">
-        <v>0</v>
-      </c>
-      <c r="G24" s="7">
-        <v>0</v>
-      </c>
-      <c r="H24" s="7">
-        <v>0</v>
-      </c>
-      <c r="I24" s="7">
-        <v>0</v>
-      </c>
-      <c r="J24" s="7">
-        <v>0</v>
-      </c>
-      <c r="K24" s="7">
-        <v>0</v>
-      </c>
-      <c r="L24" s="7">
-        <v>0</v>
-      </c>
-      <c r="M24" s="7">
-        <v>0</v>
-      </c>
-      <c r="N24" s="7">
-        <v>0</v>
-      </c>
-      <c r="O24" s="7">
-        <v>0</v>
-      </c>
-      <c r="P24" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="7">
-        <v>0</v>
-      </c>
-      <c r="R24" s="7">
-        <v>0</v>
-      </c>
-      <c r="S24" s="7">
-        <v>0</v>
-      </c>
-      <c r="T24" s="7">
-        <v>0</v>
-      </c>
-      <c r="U24" s="7">
-        <v>0</v>
-      </c>
-      <c r="V24" s="7">
-        <v>0</v>
-      </c>
-      <c r="W24" s="7">
-        <v>0</v>
-      </c>
-      <c r="X24" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ24" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR24" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="7">
-        <v>0</v>
-      </c>
-      <c r="E25" s="7">
-        <v>0</v>
-      </c>
-      <c r="F25" s="7">
-        <v>0</v>
-      </c>
-      <c r="G25" s="7">
-        <v>0</v>
-      </c>
-      <c r="H25" s="7">
-        <v>0</v>
-      </c>
-      <c r="I25" s="7">
-        <v>0</v>
-      </c>
-      <c r="J25" s="7">
-        <v>0</v>
-      </c>
-      <c r="K25" s="7">
-        <v>0</v>
-      </c>
-      <c r="L25" s="7">
-        <v>0</v>
-      </c>
-      <c r="M25" s="7">
-        <v>0</v>
-      </c>
-      <c r="N25" s="7">
-        <v>0</v>
-      </c>
-      <c r="O25" s="7">
-        <v>0</v>
-      </c>
-      <c r="P25" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="7">
-        <v>0</v>
-      </c>
-      <c r="R25" s="7">
-        <v>0</v>
-      </c>
-      <c r="S25" s="7">
-        <v>0</v>
-      </c>
-      <c r="T25" s="7">
-        <v>0</v>
-      </c>
-      <c r="U25" s="7">
-        <v>0</v>
-      </c>
-      <c r="V25" s="7">
-        <v>0</v>
-      </c>
-      <c r="W25" s="7">
-        <v>0</v>
-      </c>
-      <c r="X25" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ25" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR25" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="7">
-        <v>0</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="M26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="N26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="O26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="P26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="R26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="S26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="T26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="U26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="V26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="W26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="X26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AQ26" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR26" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D27" s="7">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <v>0</v>
-      </c>
-      <c r="F27" s="7">
-        <v>0</v>
-      </c>
-      <c r="G27" s="7">
-        <v>0</v>
-      </c>
-      <c r="H27" s="7">
-        <v>0</v>
-      </c>
-      <c r="I27" s="7">
-        <v>0</v>
-      </c>
-      <c r="J27" s="7">
-        <v>0</v>
-      </c>
-      <c r="K27" s="7">
-        <v>0</v>
-      </c>
-      <c r="L27" s="7">
-        <v>0</v>
-      </c>
-      <c r="M27" s="7">
-        <v>0</v>
-      </c>
-      <c r="N27" s="7">
-        <v>0</v>
-      </c>
-      <c r="O27" s="7">
-        <v>0</v>
-      </c>
-      <c r="P27" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="7">
-        <v>0</v>
-      </c>
-      <c r="R27" s="7">
-        <v>0</v>
-      </c>
-      <c r="S27" s="7">
-        <v>0</v>
-      </c>
-      <c r="T27" s="7">
-        <v>0</v>
-      </c>
-      <c r="U27" s="7">
-        <v>0</v>
-      </c>
-      <c r="V27" s="7">
-        <v>0</v>
-      </c>
-      <c r="W27" s="7">
-        <v>0</v>
-      </c>
-      <c r="X27" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AH27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AI27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AJ27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AK27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AL27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AM27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AN27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AO27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AP27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AQ27" s="7">
-        <v>0</v>
-      </c>
-      <c r="AR27" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>